<commit_message>
feat: expand controlled import and reporting workflows
</commit_message>
<xml_diff>
--- a/apps/project-tracker/src/ProjectTracker.Api/Assets/Templates/Project-Tracker-Controlled-Import-Template.xlsx
+++ b/apps/project-tracker/src/ProjectTracker.Api/Assets/Templates/Project-Tracker-Controlled-Import-Template.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Projects" sheetId="1" r:id="Rb9ea8aa380284cf1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Operations" sheetId="2" r:id="R0a3093684f7d4066"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Projects" sheetId="1" r:id="R54b430f7d3fb49de"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Operations" sheetId="2" r:id="Rbf5c636bdb834f03"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -3455,7 +3455,7 @@
         <x:v>Project ID (Required)</x:v>
       </x:c>
       <x:c r="B1" s="18" t="str">
-        <x:v>Operation ID (Required)</x:v>
+        <x:v>Operation ID (System)</x:v>
       </x:c>
       <x:c r="C1" s="18" t="str">
         <x:v>Sequence (Required)</x:v>

</xml_diff>

<commit_message>
feat: add enterprise sync and ITAR Fulcrum support
</commit_message>
<xml_diff>
--- a/apps/project-tracker/src/ProjectTracker.Api/Assets/Templates/Project-Tracker-Controlled-Import-Template.xlsx
+++ b/apps/project-tracker/src/ProjectTracker.Api/Assets/Templates/Project-Tracker-Controlled-Import-Template.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Projects" sheetId="1" r:id="R54b430f7d3fb49de"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Operations" sheetId="2" r:id="Rbf5c636bdb834f03"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Projects" sheetId="1" r:id="R3fa365a6747b43cf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Operations" sheetId="2" r:id="Rb21ba9d6c370484f"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -14,11 +14,12 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:numFmts count="2">
+  <x:numFmts count="3">
     <x:numFmt numFmtId="200" formatCode="yyyy-mm-dd"/>
     <x:numFmt numFmtId="201" formatCode="0%"/>
+    <x:numFmt numFmtId="202" formatCode="#,##0.####"/>
   </x:numFmts>
-  <x:fonts count="2">
+  <x:fonts count="3">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -29,8 +30,14 @@
       <x:color rgb="FFFFFFFF"/>
       <x:name val="Aptos"/>
     </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="11"/>
+      <x:color rgb="FFFFFFFF"/>
+      <x:name val="Carlito"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="4">
+  <x:fills count="5">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -45,6 +52,11 @@
     <x:fill>
       <x:patternFill patternType="solid">
         <x:fgColor rgb="FFB53A2D"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF17324D"/>
       </x:patternFill>
     </x:fill>
   </x:fills>
@@ -114,7 +126,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="22">
+  <x:cellXfs count="28">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -165,6 +177,18 @@
     </x:xf>
     <x:xf numFmtId="200" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="201" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="202" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -381,6 +405,8 @@
     <x:col min="12" max="12" width="21" hidden="0" customWidth="1"/>
     <x:col min="13" max="13" width="19" hidden="0" customWidth="1"/>
     <x:col min="14" max="14" width="26" hidden="0" customWidth="1"/>
+    <x:col min="15" max="15" width="22" hidden="0" customWidth="1"/>
+    <x:col min="16" max="16" width="28" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="34" customHeight="1">
@@ -406,41 +432,50 @@
         <x:v>Job Number</x:v>
       </x:c>
       <x:c r="H1" s="13" t="str">
+        <x:v>Required Quantity</x:v>
+      </x:c>
+      <x:c r="I1" s="13" t="str">
+        <x:v>Job Quantity</x:v>
+      </x:c>
+      <x:c r="J1" s="13" t="str">
         <x:v>Priority</x:v>
       </x:c>
-      <x:c r="I1" s="13" t="str">
+      <x:c r="K1" s="13" t="str">
         <x:v>Completed On</x:v>
       </x:c>
-      <x:c r="J1" s="13" t="str">
+      <x:c r="L1" s="13" t="str">
         <x:v>Program Start (Read Only)</x:v>
       </x:c>
-      <x:c r="K1" s="13" t="str">
+      <x:c r="M1" s="13" t="str">
         <x:v>Target Delivery (Read Only)</x:v>
       </x:c>
-      <x:c r="L1" s="13" t="str">
+      <x:c r="N1" s="14" t="str">
         <x:v>Current Status (Read Only)</x:v>
       </x:c>
-      <x:c r="M1" s="13" t="str">
+      <x:c r="O1" s="26" t="str">
         <x:v>Progress (Read Only)</x:v>
       </x:c>
-      <x:c r="N1" s="14" t="str">
+      <x:c r="P1" s="26" t="str">
         <x:v>Current Operation (Read Only)</x:v>
       </x:c>
     </x:row>
     <x:row r="2">
-      <x:c r="I2" s="20"/>
+      <x:c r="H2" s="27"/>
+      <x:c r="I2" s="27"/>
       <x:c r="J2" s="20"/>
       <x:c r="K2" s="20"/>
       <x:c r="M2" s="21"/>
     </x:row>
     <x:row r="3">
-      <x:c r="I3" s="20"/>
+      <x:c r="H3" s="27"/>
+      <x:c r="I3" s="27"/>
       <x:c r="J3" s="20"/>
       <x:c r="K3" s="20"/>
       <x:c r="M3" s="21"/>
     </x:row>
     <x:row r="4">
-      <x:c r="I4" s="20"/>
+      <x:c r="H4" s="27"/>
+      <x:c r="I4" s="27"/>
       <x:c r="J4" s="20"/>
       <x:c r="K4" s="20"/>
       <x:c r="M4" s="21"/>

</xml_diff>